<commit_message>
update the api documents
</commit_message>
<xml_diff>
--- a/api 명세서.xlsx
+++ b/api 명세서.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29822"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46DEAB72-F58D-4008-916A-EC7AC8DB8B79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{618328F0-2C74-4A14-8C9A-51CBC236CB22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="104">
   <si>
     <t>GET</t>
   </si>
@@ -71,12 +71,6 @@
     <t>전체 지역의 진행중 행사 중 좋아요순 상위 10개 조회</t>
   </si>
   <si>
-    <t>/api/events/search?keyword={keyword}&amp;limit={limit}</t>
-  </si>
-  <si>
-    <t>검색창 입력 키워드를 포함한 행사 검색 결과 조회</t>
-  </si>
-  <si>
     <t>AI</t>
   </si>
   <si>
@@ -210,9 +204,6 @@
   </si>
   <si>
     <t>/api/search?keyword={keyword}</t>
-  </si>
-  <si>
-    <t>행사 또는 관광 정보 통합 검색 결과 조회</t>
   </si>
   <si>
     <t>{ success: boolean, events: [{ content_id, title, region, first_image, start_date, end_date }] }</t>
@@ -335,6 +326,10 @@
   </si>
   <si>
     <t>/api/events/filter?region={region}&amp;status={status}&amp;lclsSystm3={lclsSystm3}&amp;start_date={start_date}&amp;end_date={end_date}&amp;keyword={keyword}</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>웹페이지 헤더 통합 검색 결과 조회</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>
@@ -373,15 +368,57 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.14999847407452621"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.749992370372631"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -389,21 +426,80 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="표준" xfId="0" builtinId="0"/>
@@ -738,7 +834,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A2:F33"/>
+  <dimension ref="A2:F32"/>
   <sheetFormatPr defaultRowHeight="16.5" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="12.625" customWidth="1"/>
@@ -749,7 +845,7 @@
     <col min="6" max="6" width="157.875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:6" ht="30" customHeight="1">
+    <row r="2" spans="1:6" s="2" customFormat="1" ht="30" customHeight="1">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -769,607 +865,587 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="30" customHeight="1">
-      <c r="A3" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="2" t="s">
+    <row r="3" spans="1:6" s="5" customFormat="1" ht="30" customHeight="1">
+      <c r="A3" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="E3" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F3" s="3" t="s">
+      <c r="E3" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="F3" s="4" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="30" customHeight="1">
-      <c r="A4" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B4" s="2" t="s">
+    <row r="4" spans="1:6" s="5" customFormat="1" ht="30" customHeight="1">
+      <c r="A4" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B4" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="D4" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="E4" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F4" s="3" t="s">
+      <c r="E4" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4" s="4" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="30" customHeight="1">
-      <c r="A5" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C5" s="3" t="s">
+    <row r="5" spans="1:6" s="8" customFormat="1" ht="30" customHeight="1">
+      <c r="A5" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="B5" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="C5" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="E5" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" ht="30" customHeight="1">
-      <c r="A6" s="2" t="s">
+      <c r="D5" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" s="8" customFormat="1" ht="30" customHeight="1">
+      <c r="A6" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="B6" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="E6" s="3" t="s">
+      <c r="B6" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C6" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="F6" s="3" t="s">
+      <c r="D6" s="6" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" ht="30" customHeight="1">
-      <c r="A7" s="2" t="s">
+      <c r="E6" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" s="11" customFormat="1" ht="30" customHeight="1">
+      <c r="A7" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="C7" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="D7" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="E7" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F7" s="10" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" s="11" customFormat="1" ht="30" customHeight="1">
+      <c r="A8" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="B7" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="E7" s="3" t="s">
+      <c r="B8" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="F7" s="3" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" ht="30" customHeight="1">
-      <c r="A8" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C8" s="3" t="s">
+      <c r="C8" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="D8" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="E8" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F8" s="3" t="s">
+      <c r="E8" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F8" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" s="11" customFormat="1" ht="30" customHeight="1">
+      <c r="A9" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="B9" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="C9" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="D9" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="E9" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F9" s="10" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" s="11" customFormat="1" ht="30" customHeight="1">
+      <c r="A10" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="B10" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="C10" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="D10" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="E10" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F10" s="10" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" s="11" customFormat="1" ht="30" customHeight="1">
+      <c r="A11" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="B11" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="C11" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="D11" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="E11" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F11" s="10" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" s="11" customFormat="1" ht="30" customHeight="1">
+      <c r="A12" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="B12" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="C12" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="D12" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="E12" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F12" s="10" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" s="11" customFormat="1" ht="30" customHeight="1">
+      <c r="A13" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="B13" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="C13" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="D13" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="E13" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="F13" s="10" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" s="11" customFormat="1" ht="30" customHeight="1">
+      <c r="A14" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="B14" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="C14" s="10" t="s">
+        <v>48</v>
+      </c>
+      <c r="D14" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="E14" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="F14" s="10" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" s="11" customFormat="1" ht="30" customHeight="1">
+      <c r="A15" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="B15" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="C15" s="10" t="s">
+        <v>48</v>
+      </c>
+      <c r="D15" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="E15" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F15" s="10" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" s="14" customFormat="1" ht="30" customHeight="1">
+      <c r="A16" s="12" t="s">
+        <v>1</v>
+      </c>
+      <c r="B16" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="C16" s="13" t="s">
+        <v>81</v>
+      </c>
+      <c r="D16" s="12" t="s">
+        <v>82</v>
+      </c>
+      <c r="E16" s="13" t="s">
+        <v>83</v>
+      </c>
+      <c r="F16" s="13" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" s="14" customFormat="1" ht="30" customHeight="1">
+      <c r="A17" s="12" t="s">
+        <v>0</v>
+      </c>
+      <c r="B17" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="C17" s="13" t="s">
+        <v>84</v>
+      </c>
+      <c r="D17" s="12" t="s">
+        <v>85</v>
+      </c>
+      <c r="E17" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="F17" s="13" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" s="14" customFormat="1" ht="30" customHeight="1">
+      <c r="A18" s="12" t="s">
+        <v>0</v>
+      </c>
+      <c r="B18" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="C18" s="13" t="s">
+        <v>87</v>
+      </c>
+      <c r="D18" s="12" t="s">
+        <v>88</v>
+      </c>
+      <c r="E18" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="F18" s="13" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" s="14" customFormat="1" ht="30" customHeight="1">
+      <c r="A19" s="12" t="s">
+        <v>1</v>
+      </c>
+      <c r="B19" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="C19" s="13" t="s">
+        <v>53</v>
+      </c>
+      <c r="D19" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="E19" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="F19" s="13" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" s="14" customFormat="1" ht="30" customHeight="1">
+      <c r="A20" s="12" t="s">
+        <v>1</v>
+      </c>
+      <c r="B20" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="C20" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="D20" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="E20" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="F20" s="13" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" s="17" customFormat="1" ht="30" customHeight="1">
+      <c r="A21" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="B21" s="15" t="s">
+        <v>61</v>
+      </c>
+      <c r="C21" s="16" t="s">
+        <v>62</v>
+      </c>
+      <c r="D21" s="15" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" ht="30" customHeight="1">
-      <c r="A9" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F9" s="3" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" ht="30" customHeight="1">
-      <c r="A10" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F10" s="3" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" ht="30" customHeight="1">
-      <c r="A11" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F11" s="3" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" ht="30" customHeight="1">
-      <c r="A12" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F12" s="3" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" ht="30" customHeight="1">
-      <c r="A13" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F13" s="3" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" ht="30" customHeight="1">
-      <c r="A14" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C14" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="E14" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="F14" s="3" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" ht="30" customHeight="1">
-      <c r="A15" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C15" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="E15" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="F15" s="3" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" ht="30" customHeight="1">
-      <c r="A16" s="2" t="s">
+      <c r="E21" s="15" t="s">
+        <v>14</v>
+      </c>
+      <c r="F21" s="16" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" s="20" customFormat="1" ht="30" customHeight="1">
+      <c r="A22" s="18" t="s">
+        <v>0</v>
+      </c>
+      <c r="B22" s="18" t="s">
+        <v>64</v>
+      </c>
+      <c r="C22" s="19" t="s">
+        <v>65</v>
+      </c>
+      <c r="D22" s="18" t="s">
+        <v>66</v>
+      </c>
+      <c r="E22" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="F22" s="19" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" s="20" customFormat="1" ht="30" customHeight="1">
+      <c r="A23" s="18" t="s">
+        <v>5</v>
+      </c>
+      <c r="B23" s="18" t="s">
+        <v>64</v>
+      </c>
+      <c r="C23" s="19" t="s">
+        <v>65</v>
+      </c>
+      <c r="D23" s="18" t="s">
+        <v>67</v>
+      </c>
+      <c r="E23" s="19" t="s">
+        <v>68</v>
+      </c>
+      <c r="F23" s="19" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" s="20" customFormat="1" ht="30" customHeight="1">
+      <c r="A24" s="18" t="s">
+        <v>0</v>
+      </c>
+      <c r="B24" s="18" t="s">
+        <v>64</v>
+      </c>
+      <c r="C24" s="19" t="s">
+        <v>69</v>
+      </c>
+      <c r="D24" s="18" t="s">
+        <v>70</v>
+      </c>
+      <c r="E24" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="F24" s="19" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" s="20" customFormat="1" ht="30" customHeight="1">
+      <c r="A25" s="18" t="s">
         <v>6</v>
       </c>
-      <c r="B16" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C16" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="D16" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="E16" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F16" s="3" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" ht="30" customHeight="1">
-      <c r="A17" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="C17" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="D17" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="E17" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="F17" s="3" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" ht="30" customHeight="1">
-      <c r="A18" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="C18" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="D18" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="E18" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="F18" s="3" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" ht="30" customHeight="1">
-      <c r="A19" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B19" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="C19" s="3" t="s">
+      <c r="B25" s="18" t="s">
         <v>64</v>
       </c>
-      <c r="D19" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="E19" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F19" s="3" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" ht="30" customHeight="1">
-      <c r="A20" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B20" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="C20" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="D20" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="E20" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F20" s="3" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" ht="30" customHeight="1">
-      <c r="A21" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B21" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="C21" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="D21" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="E21" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="F21" s="3" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" ht="30" customHeight="1">
-      <c r="A22" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B22" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="C22" s="3" t="s">
+      <c r="C25" s="19" t="s">
         <v>72</v>
       </c>
-      <c r="D22" s="2" t="s">
+      <c r="D25" s="18" t="s">
         <v>73</v>
       </c>
-      <c r="E22" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F22" s="3" t="s">
+      <c r="E25" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="F25" s="19" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="23" spans="1:6" ht="30" customHeight="1">
-      <c r="A23" s="2" t="s">
+    <row r="26" spans="1:6" s="20" customFormat="1" ht="30" customHeight="1">
+      <c r="A26" s="18" t="s">
+        <v>0</v>
+      </c>
+      <c r="B26" s="18" t="s">
+        <v>64</v>
+      </c>
+      <c r="C26" s="19" t="s">
+        <v>75</v>
+      </c>
+      <c r="D26" s="18" t="s">
+        <v>76</v>
+      </c>
+      <c r="E26" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="F26" s="19" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" s="20" customFormat="1" ht="30" customHeight="1">
+      <c r="A27" s="18" t="s">
         <v>6</v>
       </c>
-      <c r="B23" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="C23" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="D23" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="E23" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F23" s="3" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" ht="30" customHeight="1">
-      <c r="A24" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B24" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="C24" s="3" t="s">
+      <c r="B27" s="18" t="s">
+        <v>64</v>
+      </c>
+      <c r="C27" s="19" t="s">
         <v>78</v>
       </c>
-      <c r="D24" s="2" t="s">
+      <c r="D27" s="18" t="s">
         <v>79</v>
       </c>
-      <c r="E24" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F24" s="3" t="s">
+      <c r="E27" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="F27" s="19" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="25" spans="1:6" ht="30" customHeight="1">
-      <c r="A25" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B25" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="C25" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="D25" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="E25" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F25" s="3" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" ht="30" customHeight="1">
-      <c r="A26" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B26" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="C26" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="D26" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="E26" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="F26" s="3" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" ht="30" customHeight="1">
-      <c r="A27" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B27" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="C27" s="3" t="s">
-        <v>87</v>
-      </c>
-      <c r="D27" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="E27" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F27" s="3" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" ht="30" customHeight="1">
-      <c r="A28" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B28" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="C28" s="3" t="s">
+    <row r="28" spans="1:6" s="23" customFormat="1" ht="30" customHeight="1">
+      <c r="A28" s="21" t="s">
+        <v>0</v>
+      </c>
+      <c r="B28" s="21" t="s">
         <v>90</v>
       </c>
-      <c r="D28" s="2" t="s">
+      <c r="C28" s="22" t="s">
         <v>91</v>
       </c>
-      <c r="E28" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F28" s="3" t="s">
+      <c r="D28" s="21" t="s">
         <v>92</v>
       </c>
-    </row>
-    <row r="29" spans="1:6" ht="30" customHeight="1">
-      <c r="A29" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B29" s="2" t="s">
+      <c r="E28" s="21" t="s">
+        <v>14</v>
+      </c>
+      <c r="F28" s="22" t="s">
         <v>93</v>
       </c>
-      <c r="C29" s="3" t="s">
+    </row>
+    <row r="29" spans="1:6" s="23" customFormat="1" ht="30" customHeight="1">
+      <c r="A29" s="21" t="s">
+        <v>0</v>
+      </c>
+      <c r="B29" s="21" t="s">
+        <v>90</v>
+      </c>
+      <c r="C29" s="22" t="s">
+        <v>102</v>
+      </c>
+      <c r="D29" s="21" t="s">
+        <v>101</v>
+      </c>
+      <c r="E29" s="21" t="s">
+        <v>14</v>
+      </c>
+      <c r="F29" s="22" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" s="23" customFormat="1" ht="30" customHeight="1">
+      <c r="A30" s="21" t="s">
+        <v>0</v>
+      </c>
+      <c r="B30" s="21" t="s">
+        <v>90</v>
+      </c>
+      <c r="C30" s="22" t="s">
         <v>94</v>
       </c>
-      <c r="D29" s="2" t="s">
+      <c r="D30" s="21" t="s">
         <v>95</v>
       </c>
-      <c r="E29" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F29" s="3" t="s">
+      <c r="E30" s="21" t="s">
+        <v>14</v>
+      </c>
+      <c r="F30" s="22" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="30" spans="1:6" ht="30" customHeight="1">
-      <c r="A30" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B30" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="C30" s="3" t="s">
-        <v>105</v>
-      </c>
-      <c r="D30" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="E30" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F30" s="3" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6" ht="30" customHeight="1">
-      <c r="A31" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B31" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="C31" s="3" t="s">
+    <row r="31" spans="1:6" s="23" customFormat="1" ht="30" customHeight="1">
+      <c r="A31" s="21" t="s">
+        <v>0</v>
+      </c>
+      <c r="B31" s="21" t="s">
+        <v>90</v>
+      </c>
+      <c r="C31" s="22" t="s">
         <v>97</v>
       </c>
-      <c r="D31" s="2" t="s">
+      <c r="D31" s="21" t="s">
         <v>98</v>
       </c>
-      <c r="E31" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F31" s="3" t="s">
+      <c r="E31" s="21" t="s">
+        <v>14</v>
+      </c>
+      <c r="F31" s="22" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="32" spans="1:6" ht="30" customHeight="1">
-      <c r="A32" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B32" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="C32" s="3" t="s">
-        <v>100</v>
-      </c>
-      <c r="D32" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="E32" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F32" s="3" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="33" ht="30" customHeight="1"/>
+    <row r="32" spans="1:6" ht="30" customHeight="1"/>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>